<commit_message>
feat: actualizar Pulmon de Oriente v2 con datos 2025+2026, corregir busqueda VIF
</commit_message>
<xml_diff>
--- a/outputs/IMAGENES_POR_ITT/itt_pulmon_oriente/ITT_Pulmon_Oriente_2025.xlsx
+++ b/outputs/IMAGENES_POR_ITT/itt_pulmon_oriente/ITT_Pulmon_Oriente_2025.xlsx
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -47,21 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,42 +419,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>año</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>score_seguridad</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>score_cohesion</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>score_movilidad</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>score_entorno_u</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>score_educ_des</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ITT</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>nivel</t>
         </is>
@@ -480,7 +468,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>46.32</v>
+        <v>25.9</v>
       </c>
       <c r="D2" t="n">
         <v>35</v>
@@ -492,7 +480,7 @@
         <v>54.9</v>
       </c>
       <c r="G2" t="n">
-        <v>29.28</v>
+        <v>26.84</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -508,7 +496,7 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>44.77</v>
+        <v>25.9</v>
       </c>
       <c r="D3" t="n">
         <v>35</v>
@@ -520,7 +508,7 @@
         <v>54.9</v>
       </c>
       <c r="G3" t="n">
-        <v>29.1</v>
+        <v>26.84</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -536,7 +524,7 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>40.07</v>
+        <v>25.9</v>
       </c>
       <c r="D4" t="n">
         <v>35</v>
@@ -548,7 +536,7 @@
         <v>54.9</v>
       </c>
       <c r="G4" t="n">
-        <v>28.54</v>
+        <v>26.84</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -571,82 +559,82 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>año</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>trimestre</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>homicidios</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>hurtos</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>vif</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>periodo</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>score_homicidios</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>score_hurtos</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>score_vif</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>score_seguridad</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>score_cohesion</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>score_movilidad</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>score_entorno_u</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>score_educ_des</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>ITT</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>nivel</t>
         </is>
@@ -666,7 +654,7 @@
         <v>9219</v>
       </c>
       <c r="E2" t="n">
-        <v>106</v>
+        <v>1430</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -680,13 +668,13 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>67.14</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>48.28</v>
+        <v>25.9</v>
       </c>
       <c r="L2" t="n">
         <v>35</v>
@@ -698,7 +686,7 @@
         <v>54.9</v>
       </c>
       <c r="O2" t="n">
-        <v>29.52</v>
+        <v>26.84</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -720,7 +708,7 @@
         <v>9369</v>
       </c>
       <c r="E3" t="n">
-        <v>138</v>
+        <v>1728</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -734,13 +722,13 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>44.29</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>40.66</v>
+        <v>25.9</v>
       </c>
       <c r="L3" t="n">
         <v>35</v>
@@ -752,7 +740,7 @@
         <v>54.9</v>
       </c>
       <c r="O3" t="n">
-        <v>28.61</v>
+        <v>26.84</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -774,7 +762,7 @@
         <v>9422</v>
       </c>
       <c r="E4" t="n">
-        <v>125</v>
+        <v>1845</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -788,13 +776,13 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>53.57</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>43.76</v>
+        <v>25.9</v>
       </c>
       <c r="L4" t="n">
         <v>35</v>
@@ -806,7 +794,7 @@
         <v>54.9</v>
       </c>
       <c r="O4" t="n">
-        <v>28.98</v>
+        <v>26.84</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -828,7 +816,7 @@
         <v>7956</v>
       </c>
       <c r="E5" t="n">
-        <v>88</v>
+        <v>1393</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -842,13 +830,13 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>52.57</v>
+        <v>25.9</v>
       </c>
       <c r="L5" t="n">
         <v>35</v>
@@ -860,7 +848,7 @@
         <v>54.9</v>
       </c>
       <c r="O5" t="n">
-        <v>30.04</v>
+        <v>26.84</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -882,7 +870,7 @@
         <v>8217</v>
       </c>
       <c r="E6" t="n">
-        <v>98</v>
+        <v>1718</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -896,13 +884,13 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>72.86</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>50.19</v>
+        <v>25.9</v>
       </c>
       <c r="L6" t="n">
         <v>35</v>
@@ -914,7 +902,7 @@
         <v>54.9</v>
       </c>
       <c r="O6" t="n">
-        <v>29.75</v>
+        <v>26.84</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -936,7 +924,7 @@
         <v>7962</v>
       </c>
       <c r="E7" t="n">
-        <v>123</v>
+        <v>1669</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -950,13 +938,13 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>44.23</v>
+        <v>25.9</v>
       </c>
       <c r="L7" t="n">
         <v>35</v>
@@ -968,7 +956,7 @@
         <v>54.9</v>
       </c>
       <c r="O7" t="n">
-        <v>29.04</v>
+        <v>26.84</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
@@ -990,7 +978,7 @@
         <v>7811</v>
       </c>
       <c r="E8" t="n">
-        <v>136</v>
+        <v>1769</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1004,13 +992,13 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>45.71</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>41.14</v>
+        <v>25.9</v>
       </c>
       <c r="L8" t="n">
         <v>35</v>
@@ -1022,7 +1010,7 @@
         <v>54.9</v>
       </c>
       <c r="O8" t="n">
-        <v>28.66</v>
+        <v>26.84</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -1044,7 +1032,7 @@
         <v>7945</v>
       </c>
       <c r="E9" t="n">
-        <v>126</v>
+        <v>1640</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1058,13 +1046,13 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>52.86</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>43.52</v>
+        <v>25.9</v>
       </c>
       <c r="L9" t="n">
         <v>35</v>
@@ -1076,7 +1064,7 @@
         <v>54.9</v>
       </c>
       <c r="O9" t="n">
-        <v>28.95</v>
+        <v>26.84</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
@@ -1098,7 +1086,7 @@
         <v>7502</v>
       </c>
       <c r="E10" t="n">
-        <v>126</v>
+        <v>1883</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1112,13 +1100,13 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>52.86</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>43.52</v>
+        <v>25.9</v>
       </c>
       <c r="L10" t="n">
         <v>35</v>
@@ -1130,7 +1118,7 @@
         <v>54.9</v>
       </c>
       <c r="O10" t="n">
-        <v>28.95</v>
+        <v>26.84</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
@@ -1152,7 +1140,7 @@
         <v>7491</v>
       </c>
       <c r="E11" t="n">
-        <v>142</v>
+        <v>1708</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1166,13 +1154,13 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>41.43</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>39.71</v>
+        <v>25.9</v>
       </c>
       <c r="L11" t="n">
         <v>35</v>
@@ -1184,7 +1172,7 @@
         <v>54.9</v>
       </c>
       <c r="O11" t="n">
-        <v>28.49</v>
+        <v>26.84</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -1206,7 +1194,7 @@
         <v>7587</v>
       </c>
       <c r="E12" t="n">
-        <v>189</v>
+        <v>1912</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1220,13 +1208,13 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>7.86</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>28.52</v>
+        <v>25.9</v>
       </c>
       <c r="L12" t="n">
         <v>35</v>
@@ -1238,7 +1226,7 @@
         <v>54.9</v>
       </c>
       <c r="O12" t="n">
-        <v>27.15</v>
+        <v>26.84</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
@@ -1260,7 +1248,7 @@
         <v>7364</v>
       </c>
       <c r="E13" t="n">
-        <v>105</v>
+        <v>1318</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1274,13 +1262,13 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>67.86</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>48.52</v>
+        <v>25.9</v>
       </c>
       <c r="L13" t="n">
         <v>35</v>
@@ -1292,7 +1280,7 @@
         <v>54.9</v>
       </c>
       <c r="O13" t="n">
-        <v>29.55</v>
+        <v>26.84</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
@@ -1315,22 +1303,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>año</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>homicidios</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>hurtos</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>vif</t>
         </is>
@@ -1347,7 +1335,7 @@
         <v>35966</v>
       </c>
       <c r="D2" t="n">
-        <v>457</v>
+        <v>6396</v>
       </c>
     </row>
     <row r="3">
@@ -1361,7 +1349,7 @@
         <v>31935</v>
       </c>
       <c r="D3" t="n">
-        <v>483</v>
+        <v>6796</v>
       </c>
     </row>
     <row r="4">
@@ -1375,7 +1363,7 @@
         <v>29944</v>
       </c>
       <c r="D4" t="n">
-        <v>562</v>
+        <v>6821</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: actualizar .py con comparendos/rinas, eliminar parcial 2026, regenerar imagenes
</commit_message>
<xml_diff>
--- a/outputs/IMAGENES_POR_ITT/itt_pulmon_oriente/ITT_Pulmon_Oriente_2025.xlsx
+++ b/outputs/IMAGENES_POR_ITT/itt_pulmon_oriente/ITT_Pulmon_Oriente_2025.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,10 +465,10 @@
         <v>2023</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>41.01</v>
       </c>
       <c r="C2" t="n">
-        <v>25.9</v>
+        <v>42.8</v>
       </c>
       <c r="D2" t="n">
         <v>35</v>
@@ -480,11 +480,11 @@
         <v>54.9</v>
       </c>
       <c r="G2" t="n">
-        <v>26.84</v>
+        <v>41.16</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Emergencia</t>
+          <t>Consolidacion</t>
         </is>
       </c>
     </row>
@@ -493,10 +493,10 @@
         <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>51.74</v>
       </c>
       <c r="C3" t="n">
-        <v>25.9</v>
+        <v>38.63</v>
       </c>
       <c r="D3" t="n">
         <v>35</v>
@@ -508,11 +508,11 @@
         <v>54.9</v>
       </c>
       <c r="G3" t="n">
-        <v>26.84</v>
+        <v>43.89</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Emergencia</t>
+          <t>Consolidacion</t>
         </is>
       </c>
     </row>
@@ -521,10 +521,10 @@
         <v>2025</v>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>64.73999999999999</v>
       </c>
       <c r="C4" t="n">
-        <v>25.9</v>
+        <v>25.41</v>
       </c>
       <c r="D4" t="n">
         <v>35</v>
@@ -536,11 +536,39 @@
         <v>54.9</v>
       </c>
       <c r="G4" t="n">
-        <v>26.84</v>
+        <v>46.2</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Emergencia</t>
+          <t>Consolidacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" t="n">
+        <v>89.87</v>
+      </c>
+      <c r="C5" t="n">
+        <v>68.03</v>
+      </c>
+      <c r="D5" t="n">
+        <v>35</v>
+      </c>
+      <c r="E5" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="G5" t="n">
+        <v>58.85</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Consolidacion</t>
         </is>
       </c>
     </row>
@@ -555,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:R17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -586,55 +614,65 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>rinas</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>periodo</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>score_homicidios</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>score_hurtos</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>score_vif</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>score_rinas</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
         <is>
           <t>score_seguridad</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>score_cohesion</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>score_movilidad</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>score_entorno_u</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>score_educ_des</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>ITT</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>nivel</t>
         </is>
@@ -648,47 +686,53 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>257</v>
+        <v>24</v>
       </c>
       <c r="D2" t="n">
-        <v>9219</v>
+        <v>431</v>
       </c>
       <c r="E2" t="n">
-        <v>1430</v>
-      </c>
-      <c r="F2" t="inlineStr">
+        <v>1360</v>
+      </c>
+      <c r="F2" t="n">
+        <v>70</v>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>2023-Q1</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>57.78</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>7.6</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>25.9</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="L2" t="n">
-        <v>35</v>
+        <v>32.69</v>
       </c>
       <c r="M2" t="n">
-        <v>39.2</v>
+        <v>39.46</v>
       </c>
       <c r="N2" t="n">
-        <v>54.9</v>
+        <v>35</v>
       </c>
       <c r="O2" t="n">
-        <v>26.84</v>
-      </c>
-      <c r="P2" t="inlineStr">
+        <v>39.2</v>
+      </c>
+      <c r="P2" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>38.27</v>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>Emergencia</t>
         </is>
@@ -702,49 +746,55 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>258</v>
+        <v>24</v>
       </c>
       <c r="D3" t="n">
-        <v>9369</v>
+        <v>373</v>
       </c>
       <c r="E3" t="n">
-        <v>1728</v>
-      </c>
-      <c r="F3" t="inlineStr">
+        <v>1658</v>
+      </c>
+      <c r="F3" t="n">
+        <v>67</v>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>2023-Q2</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>57.78</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>30.8</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>25.9</v>
+        <v>66.43000000000001</v>
       </c>
       <c r="L3" t="n">
-        <v>35</v>
+        <v>44.29</v>
       </c>
       <c r="M3" t="n">
-        <v>39.2</v>
+        <v>40.18</v>
       </c>
       <c r="N3" t="n">
-        <v>54.9</v>
+        <v>35</v>
       </c>
       <c r="O3" t="n">
-        <v>26.84</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Emergencia</t>
+        <v>39.2</v>
+      </c>
+      <c r="P3" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>41.83</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Consolidacion</t>
         </is>
       </c>
     </row>
@@ -756,47 +806,53 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>255</v>
+        <v>38</v>
       </c>
       <c r="D4" t="n">
-        <v>9422</v>
+        <v>378</v>
       </c>
       <c r="E4" t="n">
-        <v>1845</v>
-      </c>
-      <c r="F4" t="inlineStr">
+        <v>1759</v>
+      </c>
+      <c r="F4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>2023-Q3</t>
         </is>
       </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>26.67</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>28.8</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>25.9</v>
+        <v>78.56999999999999</v>
       </c>
       <c r="L4" t="n">
-        <v>35</v>
+        <v>27.73</v>
       </c>
       <c r="M4" t="n">
-        <v>39.2</v>
+        <v>44.22</v>
       </c>
       <c r="N4" t="n">
-        <v>54.9</v>
+        <v>35</v>
       </c>
       <c r="O4" t="n">
-        <v>26.84</v>
-      </c>
-      <c r="P4" t="inlineStr">
+        <v>39.2</v>
+      </c>
+      <c r="P4" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>37.35</v>
+      </c>
+      <c r="R4" t="inlineStr">
         <is>
           <t>Emergencia</t>
         </is>
@@ -810,49 +866,55 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>243</v>
+        <v>31</v>
       </c>
       <c r="D5" t="n">
-        <v>7956</v>
+        <v>259</v>
       </c>
       <c r="E5" t="n">
-        <v>1393</v>
-      </c>
-      <c r="F5" t="inlineStr">
+        <v>1340</v>
+      </c>
+      <c r="F5" t="n">
+        <v>37</v>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>2023-Q4</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>42.22</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>25.9</v>
+        <v>87.86</v>
       </c>
       <c r="L5" t="n">
-        <v>35</v>
+        <v>59.31</v>
       </c>
       <c r="M5" t="n">
-        <v>39.2</v>
+        <v>47.32</v>
       </c>
       <c r="N5" t="n">
-        <v>54.9</v>
+        <v>35</v>
       </c>
       <c r="O5" t="n">
-        <v>26.84</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Emergencia</t>
+        <v>39.2</v>
+      </c>
+      <c r="P5" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Consolidacion</t>
         </is>
       </c>
     </row>
@@ -864,49 +926,55 @@
         <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>199</v>
+        <v>18</v>
       </c>
       <c r="D6" t="n">
-        <v>8217</v>
+        <v>375</v>
       </c>
       <c r="E6" t="n">
-        <v>1718</v>
-      </c>
-      <c r="F6" t="inlineStr">
+        <v>1657</v>
+      </c>
+      <c r="F6" t="n">
+        <v>86</v>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>2024-Q1</t>
         </is>
       </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>71.11</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>25.9</v>
+        <v>52.86</v>
       </c>
       <c r="L6" t="n">
-        <v>35</v>
+        <v>50.56</v>
       </c>
       <c r="M6" t="n">
-        <v>39.2</v>
+        <v>35.65</v>
       </c>
       <c r="N6" t="n">
-        <v>54.9</v>
+        <v>35</v>
       </c>
       <c r="O6" t="n">
-        <v>26.84</v>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Emergencia</t>
+        <v>39.2</v>
+      </c>
+      <c r="P6" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>43.17</v>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Consolidacion</t>
         </is>
       </c>
     </row>
@@ -918,49 +986,55 @@
         <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>226</v>
+        <v>21</v>
       </c>
       <c r="D7" t="n">
-        <v>7962</v>
+        <v>353</v>
       </c>
       <c r="E7" t="n">
-        <v>1669</v>
-      </c>
-      <c r="F7" t="inlineStr">
+        <v>1586</v>
+      </c>
+      <c r="F7" t="n">
+        <v>91</v>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>2024-Q2</t>
         </is>
       </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>64.44</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>38.8</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>25.9</v>
+        <v>49.29</v>
       </c>
       <c r="L7" t="n">
-        <v>35</v>
+        <v>51.62</v>
       </c>
       <c r="M7" t="n">
-        <v>39.2</v>
+        <v>34.46</v>
       </c>
       <c r="N7" t="n">
-        <v>54.9</v>
+        <v>35</v>
       </c>
       <c r="O7" t="n">
-        <v>26.84</v>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Emergencia</t>
+        <v>39.2</v>
+      </c>
+      <c r="P7" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>43.35</v>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Consolidacion</t>
         </is>
       </c>
     </row>
@@ -972,49 +1046,55 @@
         <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>265</v>
+        <v>26</v>
       </c>
       <c r="D8" t="n">
-        <v>7811</v>
+        <v>349</v>
       </c>
       <c r="E8" t="n">
-        <v>1769</v>
-      </c>
-      <c r="F8" t="inlineStr">
+        <v>1712</v>
+      </c>
+      <c r="F8" t="n">
+        <v>55</v>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>2024-Q3</t>
         </is>
       </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>53.33</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>40.4</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>25.9</v>
+        <v>75</v>
       </c>
       <c r="L8" t="n">
-        <v>35</v>
+        <v>46.87</v>
       </c>
       <c r="M8" t="n">
-        <v>39.2</v>
+        <v>43.03</v>
       </c>
       <c r="N8" t="n">
-        <v>54.9</v>
+        <v>35</v>
       </c>
       <c r="O8" t="n">
-        <v>26.84</v>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>Emergencia</t>
+        <v>39.2</v>
+      </c>
+      <c r="P8" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>42.95</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Consolidacion</t>
         </is>
       </c>
     </row>
@@ -1026,49 +1106,55 @@
         <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>248</v>
+        <v>20</v>
       </c>
       <c r="D9" t="n">
-        <v>7945</v>
+        <v>327</v>
       </c>
       <c r="E9" t="n">
-        <v>1640</v>
-      </c>
-      <c r="F9" t="inlineStr">
+        <v>1545</v>
+      </c>
+      <c r="F9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>2024-Q4</t>
         </is>
       </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>66.67</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>49.2</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>25.9</v>
+        <v>70</v>
       </c>
       <c r="L9" t="n">
-        <v>35</v>
+        <v>57.93</v>
       </c>
       <c r="M9" t="n">
-        <v>39.2</v>
+        <v>41.37</v>
       </c>
       <c r="N9" t="n">
-        <v>54.9</v>
+        <v>35</v>
       </c>
       <c r="O9" t="n">
-        <v>26.84</v>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Emergencia</t>
+        <v>39.2</v>
+      </c>
+      <c r="P9" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>46.07</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Consolidacion</t>
         </is>
       </c>
     </row>
@@ -1080,49 +1166,55 @@
         <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>254</v>
+        <v>25</v>
       </c>
       <c r="D10" t="n">
-        <v>7502</v>
+        <v>287</v>
       </c>
       <c r="E10" t="n">
-        <v>1883</v>
-      </c>
-      <c r="F10" t="inlineStr">
+        <v>1785</v>
+      </c>
+      <c r="F10" t="n">
+        <v>92</v>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>2025-Q1</t>
         </is>
       </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>55.56</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>65.2</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>25.9</v>
+        <v>48.57</v>
       </c>
       <c r="L10" t="n">
-        <v>35</v>
+        <v>60.38</v>
       </c>
       <c r="M10" t="n">
-        <v>39.2</v>
+        <v>34.22</v>
       </c>
       <c r="N10" t="n">
-        <v>54.9</v>
+        <v>35</v>
       </c>
       <c r="O10" t="n">
-        <v>26.84</v>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>Emergencia</t>
+        <v>39.2</v>
+      </c>
+      <c r="P10" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>45.95</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Consolidacion</t>
         </is>
       </c>
     </row>
@@ -1134,49 +1226,55 @@
         <v>2</v>
       </c>
       <c r="C11" t="n">
-        <v>243</v>
+        <v>14</v>
       </c>
       <c r="D11" t="n">
-        <v>7491</v>
+        <v>306</v>
       </c>
       <c r="E11" t="n">
-        <v>1708</v>
-      </c>
-      <c r="F11" t="inlineStr">
+        <v>1647</v>
+      </c>
+      <c r="F11" t="n">
+        <v>120</v>
+      </c>
+      <c r="G11" t="inlineStr">
         <is>
           <t>2025-Q2</t>
         </is>
       </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>57.6</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>25.9</v>
+        <v>28.57</v>
       </c>
       <c r="L11" t="n">
-        <v>35</v>
+        <v>68.8</v>
       </c>
       <c r="M11" t="n">
-        <v>39.2</v>
+        <v>27.56</v>
       </c>
       <c r="N11" t="n">
-        <v>54.9</v>
+        <v>35</v>
       </c>
       <c r="O11" t="n">
-        <v>26.84</v>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>Emergencia</t>
+        <v>39.2</v>
+      </c>
+      <c r="P11" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>47.67</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Consolidacion</t>
         </is>
       </c>
     </row>
@@ -1188,49 +1286,55 @@
         <v>3</v>
       </c>
       <c r="C12" t="n">
-        <v>253</v>
+        <v>9</v>
       </c>
       <c r="D12" t="n">
-        <v>7587</v>
+        <v>291</v>
       </c>
       <c r="E12" t="n">
-        <v>1912</v>
-      </c>
-      <c r="F12" t="inlineStr">
+        <v>1831</v>
+      </c>
+      <c r="F12" t="n">
+        <v>144</v>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>2025-Q3</t>
         </is>
       </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>91.11</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>63.6</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>25.9</v>
+        <v>11.43</v>
       </c>
       <c r="L12" t="n">
-        <v>35</v>
+        <v>77.36</v>
       </c>
       <c r="M12" t="n">
-        <v>39.2</v>
+        <v>21.84</v>
       </c>
       <c r="N12" t="n">
-        <v>54.9</v>
+        <v>35</v>
       </c>
       <c r="O12" t="n">
-        <v>26.84</v>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>Emergencia</t>
+        <v>39.2</v>
+      </c>
+      <c r="P12" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>49.55</v>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Consolidacion</t>
         </is>
       </c>
     </row>
@@ -1242,49 +1346,295 @@
         <v>4</v>
       </c>
       <c r="C13" t="n">
-        <v>312</v>
+        <v>37</v>
       </c>
       <c r="D13" t="n">
-        <v>7364</v>
+        <v>260</v>
       </c>
       <c r="E13" t="n">
-        <v>1318</v>
-      </c>
-      <c r="F13" t="inlineStr">
+        <v>1255</v>
+      </c>
+      <c r="F13" t="n">
+        <v>243</v>
+      </c>
+      <c r="G13" t="inlineStr">
         <is>
           <t>2025-Q4</t>
         </is>
       </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>28.89</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>25.9</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>35</v>
+        <v>52.44</v>
       </c>
       <c r="M13" t="n">
-        <v>39.2</v>
+        <v>18.03</v>
       </c>
       <c r="N13" t="n">
-        <v>54.9</v>
+        <v>35</v>
       </c>
       <c r="O13" t="n">
-        <v>26.84</v>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>Emergencia</t>
+        <v>39.2</v>
+      </c>
+      <c r="P13" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>41.62</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Consolidacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>26</v>
+      </c>
+      <c r="D14" t="n">
+        <v>286</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1377</v>
+      </c>
+      <c r="F14" t="n">
+        <v>202</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-Q1</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>53.33</v>
+      </c>
+      <c r="I14" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>59.47</v>
+      </c>
+      <c r="M14" t="n">
+        <v>18.03</v>
+      </c>
+      <c r="N14" t="n">
+        <v>35</v>
+      </c>
+      <c r="O14" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="P14" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Consolidacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-Q2</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>100</v>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="n">
+        <v>100</v>
+      </c>
+      <c r="K15" t="n">
+        <v>100</v>
+      </c>
+      <c r="L15" t="n">
+        <v>100</v>
+      </c>
+      <c r="M15" t="n">
+        <v>84.7</v>
+      </c>
+      <c r="N15" t="n">
+        <v>35</v>
+      </c>
+      <c r="O15" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="P15" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>63.89</v>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Avance</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-Q3</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>100</v>
+      </c>
+      <c r="I16" t="n">
+        <v>100</v>
+      </c>
+      <c r="J16" t="n">
+        <v>100</v>
+      </c>
+      <c r="K16" t="n">
+        <v>100</v>
+      </c>
+      <c r="L16" t="n">
+        <v>100</v>
+      </c>
+      <c r="M16" t="n">
+        <v>84.7</v>
+      </c>
+      <c r="N16" t="n">
+        <v>35</v>
+      </c>
+      <c r="O16" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="P16" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>63.89</v>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Avance</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-Q4</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>100</v>
+      </c>
+      <c r="I17" t="n">
+        <v>100</v>
+      </c>
+      <c r="J17" t="n">
+        <v>100</v>
+      </c>
+      <c r="K17" t="n">
+        <v>100</v>
+      </c>
+      <c r="L17" t="n">
+        <v>100</v>
+      </c>
+      <c r="M17" t="n">
+        <v>84.7</v>
+      </c>
+      <c r="N17" t="n">
+        <v>35</v>
+      </c>
+      <c r="O17" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="P17" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>63.89</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Avance</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1323,19 +1673,27 @@
           <t>vif</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>rinas</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>2023</v>
       </c>
       <c r="B2" t="n">
-        <v>1013</v>
+        <v>117</v>
       </c>
       <c r="C2" t="n">
-        <v>35966</v>
+        <v>1441</v>
       </c>
       <c r="D2" t="n">
-        <v>6396</v>
+        <v>6117</v>
+      </c>
+      <c r="E2" t="n">
+        <v>224</v>
       </c>
     </row>
     <row r="3">
@@ -1343,13 +1701,16 @@
         <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>938</v>
+        <v>85</v>
       </c>
       <c r="C3" t="n">
-        <v>31935</v>
+        <v>1404</v>
       </c>
       <c r="D3" t="n">
-        <v>6796</v>
+        <v>6500</v>
+      </c>
+      <c r="E3" t="n">
+        <v>294</v>
       </c>
     </row>
     <row r="4">
@@ -1357,13 +1718,33 @@
         <v>2025</v>
       </c>
       <c r="B4" t="n">
-        <v>1062</v>
+        <v>85</v>
       </c>
       <c r="C4" t="n">
-        <v>29944</v>
+        <v>1144</v>
       </c>
       <c r="D4" t="n">
-        <v>6821</v>
+        <v>6518</v>
+      </c>
+      <c r="E4" t="n">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" t="n">
+        <v>26</v>
+      </c>
+      <c r="C5" t="n">
+        <v>286</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1377</v>
+      </c>
+      <c r="E5" t="n">
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Implementar valores Proxy Q2-Q4 2026 y actualizar toda la documentacion .md
</commit_message>
<xml_diff>
--- a/outputs/IMAGENES_POR_ITT/itt_pulmon_oriente/ITT_Pulmon_Oriente_2025.xlsx
+++ b/outputs/IMAGENES_POR_ITT/itt_pulmon_oriente/ITT_Pulmon_Oriente_2025.xlsx
@@ -468,7 +468,7 @@
         <v>41.01</v>
       </c>
       <c r="C2" t="n">
-        <v>42.8</v>
+        <v>63.21</v>
       </c>
       <c r="D2" t="n">
         <v>35</v>
@@ -480,7 +480,7 @@
         <v>54.9</v>
       </c>
       <c r="G2" t="n">
-        <v>41.16</v>
+        <v>43.61</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -496,7 +496,7 @@
         <v>51.74</v>
       </c>
       <c r="C3" t="n">
-        <v>38.63</v>
+        <v>57.5</v>
       </c>
       <c r="D3" t="n">
         <v>35</v>
@@ -508,7 +508,7 @@
         <v>54.9</v>
       </c>
       <c r="G3" t="n">
-        <v>43.89</v>
+        <v>46.15</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         <v>64.73999999999999</v>
       </c>
       <c r="C4" t="n">
-        <v>25.41</v>
+        <v>39.58</v>
       </c>
       <c r="D4" t="n">
         <v>35</v>
@@ -536,7 +536,7 @@
         <v>54.9</v>
       </c>
       <c r="G4" t="n">
-        <v>46.2</v>
+        <v>47.9</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -552,7 +552,7 @@
         <v>89.87</v>
       </c>
       <c r="C5" t="n">
-        <v>68.03</v>
+        <v>73.20999999999999</v>
       </c>
       <c r="D5" t="n">
         <v>35</v>
@@ -564,7 +564,7 @@
         <v>54.9</v>
       </c>
       <c r="G5" t="n">
-        <v>58.85</v>
+        <v>59.47</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -692,7 +692,7 @@
         <v>431</v>
       </c>
       <c r="E2" t="n">
-        <v>1360</v>
+        <v>106</v>
       </c>
       <c r="F2" t="n">
         <v>70</v>
@@ -709,7 +709,7 @@
         <v>7.6</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>67.14</v>
       </c>
       <c r="K2" t="n">
         <v>64.29000000000001</v>
@@ -718,7 +718,7 @@
         <v>32.69</v>
       </c>
       <c r="M2" t="n">
-        <v>39.46</v>
+        <v>61.84</v>
       </c>
       <c r="N2" t="n">
         <v>35</v>
@@ -730,11 +730,11 @@
         <v>54.9</v>
       </c>
       <c r="Q2" t="n">
-        <v>38.27</v>
+        <v>40.95</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Emergencia</t>
+          <t>Consolidacion</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
         <v>373</v>
       </c>
       <c r="E3" t="n">
-        <v>1658</v>
+        <v>138</v>
       </c>
       <c r="F3" t="n">
         <v>67</v>
@@ -769,7 +769,7 @@
         <v>30.8</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>44.29</v>
       </c>
       <c r="K3" t="n">
         <v>66.43000000000001</v>
@@ -778,7 +778,7 @@
         <v>44.29</v>
       </c>
       <c r="M3" t="n">
-        <v>40.18</v>
+        <v>54.94</v>
       </c>
       <c r="N3" t="n">
         <v>35</v>
@@ -790,7 +790,7 @@
         <v>54.9</v>
       </c>
       <c r="Q3" t="n">
-        <v>41.83</v>
+        <v>43.61</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -812,7 +812,7 @@
         <v>378</v>
       </c>
       <c r="E4" t="n">
-        <v>1759</v>
+        <v>125</v>
       </c>
       <c r="F4" t="n">
         <v>50</v>
@@ -829,7 +829,7 @@
         <v>28.8</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>53.57</v>
       </c>
       <c r="K4" t="n">
         <v>78.56999999999999</v>
@@ -838,7 +838,7 @@
         <v>27.73</v>
       </c>
       <c r="M4" t="n">
-        <v>44.22</v>
+        <v>62.08</v>
       </c>
       <c r="N4" t="n">
         <v>35</v>
@@ -850,7 +850,7 @@
         <v>54.9</v>
       </c>
       <c r="Q4" t="n">
-        <v>37.35</v>
+        <v>39.5</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -872,7 +872,7 @@
         <v>259</v>
       </c>
       <c r="E5" t="n">
-        <v>1340</v>
+        <v>88</v>
       </c>
       <c r="F5" t="n">
         <v>37</v>
@@ -889,7 +889,7 @@
         <v>76.40000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="K5" t="n">
         <v>87.86</v>
@@ -898,7 +898,7 @@
         <v>59.31</v>
       </c>
       <c r="M5" t="n">
-        <v>47.32</v>
+        <v>73.98999999999999</v>
       </c>
       <c r="N5" t="n">
         <v>35</v>
@@ -910,7 +910,7 @@
         <v>54.9</v>
       </c>
       <c r="Q5" t="n">
-        <v>47.2</v>
+        <v>50.4</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -932,7 +932,7 @@
         <v>375</v>
       </c>
       <c r="E6" t="n">
-        <v>1657</v>
+        <v>98</v>
       </c>
       <c r="F6" t="n">
         <v>86</v>
@@ -949,7 +949,7 @@
         <v>30</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>72.86</v>
       </c>
       <c r="K6" t="n">
         <v>52.86</v>
@@ -958,7 +958,7 @@
         <v>50.56</v>
       </c>
       <c r="M6" t="n">
-        <v>35.65</v>
+        <v>59.94</v>
       </c>
       <c r="N6" t="n">
         <v>35</v>
@@ -970,7 +970,7 @@
         <v>54.9</v>
       </c>
       <c r="Q6" t="n">
-        <v>43.17</v>
+        <v>46.09</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -992,7 +992,7 @@
         <v>353</v>
       </c>
       <c r="E7" t="n">
-        <v>1586</v>
+        <v>123</v>
       </c>
       <c r="F7" t="n">
         <v>91</v>
@@ -1009,7 +1009,7 @@
         <v>38.8</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="K7" t="n">
         <v>49.29</v>
@@ -1018,7 +1018,7 @@
         <v>51.62</v>
       </c>
       <c r="M7" t="n">
-        <v>34.46</v>
+        <v>52.8</v>
       </c>
       <c r="N7" t="n">
         <v>35</v>
@@ -1030,7 +1030,7 @@
         <v>54.9</v>
       </c>
       <c r="Q7" t="n">
-        <v>43.35</v>
+        <v>45.55</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
         <v>349</v>
       </c>
       <c r="E8" t="n">
-        <v>1712</v>
+        <v>136</v>
       </c>
       <c r="F8" t="n">
         <v>55</v>
@@ -1069,7 +1069,7 @@
         <v>40.4</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>45.71</v>
       </c>
       <c r="K8" t="n">
         <v>75</v>
@@ -1078,7 +1078,7 @@
         <v>46.87</v>
       </c>
       <c r="M8" t="n">
-        <v>43.03</v>
+        <v>58.27</v>
       </c>
       <c r="N8" t="n">
         <v>35</v>
@@ -1090,7 +1090,7 @@
         <v>54.9</v>
       </c>
       <c r="Q8" t="n">
-        <v>42.95</v>
+        <v>44.78</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
         <v>327</v>
       </c>
       <c r="E9" t="n">
-        <v>1545</v>
+        <v>126</v>
       </c>
       <c r="F9" t="n">
         <v>62</v>
@@ -1129,7 +1129,7 @@
         <v>49.2</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>52.86</v>
       </c>
       <c r="K9" t="n">
         <v>70</v>
@@ -1138,7 +1138,7 @@
         <v>57.93</v>
       </c>
       <c r="M9" t="n">
-        <v>41.37</v>
+        <v>58.99</v>
       </c>
       <c r="N9" t="n">
         <v>35</v>
@@ -1150,7 +1150,7 @@
         <v>54.9</v>
       </c>
       <c r="Q9" t="n">
-        <v>46.07</v>
+        <v>48.19</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -1172,7 +1172,7 @@
         <v>287</v>
       </c>
       <c r="E10" t="n">
-        <v>1785</v>
+        <v>126</v>
       </c>
       <c r="F10" t="n">
         <v>92</v>
@@ -1189,7 +1189,7 @@
         <v>65.2</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>52.86</v>
       </c>
       <c r="K10" t="n">
         <v>48.57</v>
@@ -1198,7 +1198,7 @@
         <v>60.38</v>
       </c>
       <c r="M10" t="n">
-        <v>34.22</v>
+        <v>51.84</v>
       </c>
       <c r="N10" t="n">
         <v>35</v>
@@ -1210,7 +1210,7 @@
         <v>54.9</v>
       </c>
       <c r="Q10" t="n">
-        <v>45.95</v>
+        <v>48.06</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -1232,7 +1232,7 @@
         <v>306</v>
       </c>
       <c r="E11" t="n">
-        <v>1647</v>
+        <v>142</v>
       </c>
       <c r="F11" t="n">
         <v>120</v>
@@ -1249,7 +1249,7 @@
         <v>57.6</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>41.43</v>
       </c>
       <c r="K11" t="n">
         <v>28.57</v>
@@ -1258,7 +1258,7 @@
         <v>68.8</v>
       </c>
       <c r="M11" t="n">
-        <v>27.56</v>
+        <v>41.37</v>
       </c>
       <c r="N11" t="n">
         <v>35</v>
@@ -1270,7 +1270,7 @@
         <v>54.9</v>
       </c>
       <c r="Q11" t="n">
-        <v>47.67</v>
+        <v>49.33</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -1292,7 +1292,7 @@
         <v>291</v>
       </c>
       <c r="E12" t="n">
-        <v>1831</v>
+        <v>189</v>
       </c>
       <c r="F12" t="n">
         <v>144</v>
@@ -1309,7 +1309,7 @@
         <v>63.6</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>7.86</v>
       </c>
       <c r="K12" t="n">
         <v>11.43</v>
@@ -1318,7 +1318,7 @@
         <v>77.36</v>
       </c>
       <c r="M12" t="n">
-        <v>21.84</v>
+        <v>24.46</v>
       </c>
       <c r="N12" t="n">
         <v>35</v>
@@ -1330,7 +1330,7 @@
         <v>54.9</v>
       </c>
       <c r="Q12" t="n">
-        <v>49.55</v>
+        <v>49.87</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -1352,7 +1352,7 @@
         <v>260</v>
       </c>
       <c r="E13" t="n">
-        <v>1255</v>
+        <v>105</v>
       </c>
       <c r="F13" t="n">
         <v>243</v>
@@ -1369,7 +1369,7 @@
         <v>76</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>67.86</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -1378,7 +1378,7 @@
         <v>52.44</v>
       </c>
       <c r="M13" t="n">
-        <v>18.03</v>
+        <v>40.65</v>
       </c>
       <c r="N13" t="n">
         <v>35</v>
@@ -1390,7 +1390,7 @@
         <v>54.9</v>
       </c>
       <c r="Q13" t="n">
-        <v>41.62</v>
+        <v>44.34</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -1412,7 +1412,7 @@
         <v>286</v>
       </c>
       <c r="E14" t="n">
-        <v>1377</v>
+        <v>113</v>
       </c>
       <c r="F14" t="n">
         <v>202</v>
@@ -1429,7 +1429,7 @@
         <v>65.59999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>62.14</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -1438,7 +1438,7 @@
         <v>59.47</v>
       </c>
       <c r="M14" t="n">
-        <v>18.03</v>
+        <v>38.75</v>
       </c>
       <c r="N14" t="n">
         <v>35</v>
@@ -1450,7 +1450,7 @@
         <v>54.9</v>
       </c>
       <c r="Q14" t="n">
-        <v>43.73</v>
+        <v>46.22</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>1441</v>
       </c>
       <c r="D2" t="n">
-        <v>6117</v>
+        <v>457</v>
       </c>
       <c r="E2" t="n">
         <v>224</v>
@@ -1707,7 +1707,7 @@
         <v>1404</v>
       </c>
       <c r="D3" t="n">
-        <v>6500</v>
+        <v>483</v>
       </c>
       <c r="E3" t="n">
         <v>294</v>
@@ -1724,7 +1724,7 @@
         <v>1144</v>
       </c>
       <c r="D4" t="n">
-        <v>6518</v>
+        <v>562</v>
       </c>
       <c r="E4" t="n">
         <v>599</v>
@@ -1741,7 +1741,7 @@
         <v>286</v>
       </c>
       <c r="D5" t="n">
-        <v>1377</v>
+        <v>113</v>
       </c>
       <c r="E5" t="n">
         <v>202</v>

</xml_diff>